<commit_message>
feat: completar autoría, licencia y validaciones de etapa 1
</commit_message>
<xml_diff>
--- a/realstep-head/catalog/products.xlsx
+++ b/realstep-head/catalog/products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c262efc70aa72104/Documents/catalogo_head/Catalogo_Head/realstep-head/catalog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1856" documentId="11_ADE01E1E62D19FE47686E5DB2F4B9CE89BB4BB42" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{275D5430-E245-450D-8E4E-00CF3FB95A93}"/>
+  <xr:revisionPtr revIDLastSave="1859" documentId="11_ADE01E1E62D19FE47686E5DB2F4B9CE89BB4BB42" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08025060-A83F-4BC4-9CB1-19BF296D40D9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categorias" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6553" uniqueCount="1201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6561" uniqueCount="1201">
   <si>
     <t>producto_id</t>
   </si>
@@ -13457,7 +13457,7 @@
         <v>1175</v>
       </c>
       <c r="C115" s="14" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="D115" s="14"/>
       <c r="E115" s="14"/>

</xml_diff>